<commit_message>
feat: implement organizational hierarchy model
Add Empresa, CentroCosto, and PuntoVenta entities to support granular organizational structuring. Update payroll types, service layer, and UI components to integrate these new levels into shifts and client reports.
</commit_message>
<xml_diff>
--- a/public/Plantilla_Carga_Masiva_Turnos_SERGEM.xlsx
+++ b/public/Plantilla_Carga_Masiva_Turnos_SERGEM.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT3"/>
+  <dimension ref="A1:BA3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -409,43 +409,50 @@
     <col min="7" max="7" width="9.83203125" customWidth="1"/>
     <col min="8" max="8" width="9.83203125" customWidth="1"/>
     <col min="9" max="9" width="9.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="24.83203125" customWidth="1"/>
-    <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
     <col min="13" max="13" width="9.83203125" customWidth="1"/>
     <col min="14" max="14" width="9.83203125" customWidth="1"/>
     <col min="15" max="15" width="9.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="24.83203125" customWidth="1"/>
-    <col min="18" max="18" width="9.83203125" customWidth="1"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="9.83203125" customWidth="1"/>
+    <col min="17" max="17" width="28.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="24.83203125" customWidth="1"/>
     <col min="20" max="20" width="9.83203125" customWidth="1"/>
     <col min="21" max="21" width="9.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
-    <col min="23" max="23" width="24.83203125" customWidth="1"/>
-    <col min="24" max="24" width="9.83203125" customWidth="1"/>
-    <col min="25" max="25" width="9.83203125" customWidth="1"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1"/>
+    <col min="23" max="23" width="9.83203125" customWidth="1"/>
+    <col min="24" max="24" width="28.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
+    <col min="26" max="26" width="24.83203125" customWidth="1"/>
     <col min="27" max="27" width="9.83203125" customWidth="1"/>
-    <col min="28" max="28" width="12.83203125" customWidth="1"/>
-    <col min="29" max="29" width="24.83203125" customWidth="1"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1"/>
+    <col min="29" max="29" width="9.83203125" customWidth="1"/>
     <col min="30" max="30" width="9.83203125" customWidth="1"/>
-    <col min="31" max="31" width="9.83203125" customWidth="1"/>
-    <col min="32" max="32" width="9.83203125" customWidth="1"/>
-    <col min="33" max="33" width="9.83203125" customWidth="1"/>
-    <col min="34" max="34" width="12.83203125" customWidth="1"/>
-    <col min="35" max="35" width="24.83203125" customWidth="1"/>
+    <col min="31" max="31" width="28.83203125" customWidth="1"/>
+    <col min="32" max="32" width="12.83203125" customWidth="1"/>
+    <col min="33" max="33" width="24.83203125" customWidth="1"/>
+    <col min="34" max="34" width="9.83203125" customWidth="1"/>
+    <col min="35" max="35" width="9.83203125" customWidth="1"/>
     <col min="36" max="36" width="9.83203125" customWidth="1"/>
     <col min="37" max="37" width="9.83203125" customWidth="1"/>
-    <col min="38" max="38" width="9.83203125" customWidth="1"/>
-    <col min="39" max="39" width="9.83203125" customWidth="1"/>
-    <col min="40" max="40" width="12.83203125" customWidth="1"/>
-    <col min="41" max="41" width="24.83203125" customWidth="1"/>
+    <col min="38" max="38" width="28.83203125" customWidth="1"/>
+    <col min="39" max="39" width="12.83203125" customWidth="1"/>
+    <col min="40" max="40" width="24.83203125" customWidth="1"/>
+    <col min="41" max="41" width="9.83203125" customWidth="1"/>
     <col min="42" max="42" width="9.83203125" customWidth="1"/>
     <col min="43" max="43" width="9.83203125" customWidth="1"/>
     <col min="44" max="44" width="9.83203125" customWidth="1"/>
-    <col min="45" max="45" width="9.83203125" customWidth="1"/>
-    <col min="46" max="46" width="30.83203125" customWidth="1"/>
+    <col min="45" max="45" width="28.83203125" customWidth="1"/>
+    <col min="46" max="46" width="12.83203125" customWidth="1"/>
+    <col min="47" max="47" width="24.83203125" customWidth="1"/>
+    <col min="48" max="48" width="9.83203125" customWidth="1"/>
+    <col min="49" max="49" width="9.83203125" customWidth="1"/>
+    <col min="50" max="50" width="9.83203125" customWidth="1"/>
+    <col min="51" max="51" width="9.83203125" customWidth="1"/>
+    <col min="52" max="52" width="28.83203125" customWidth="1"/>
+    <col min="53" max="53" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,115 +484,136 @@
         <v>Lunes_Fin2</v>
       </c>
       <c r="J1" t="str">
+        <v>Lunes_Observaciones</v>
+      </c>
+      <c r="K1" t="str">
         <v>Martes_Tipo</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Martes_Cliente</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Martes_Inicio1</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Martes_Fin1</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Martes_Inicio2</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Martes_Fin2</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
+        <v>Martes_Observaciones</v>
+      </c>
+      <c r="R1" t="str">
         <v>Miercoles_Tipo</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>Miercoles_Cliente</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>Miercoles_Inicio1</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>Miercoles_Fin1</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Miercoles_Inicio2</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Miercoles_Fin2</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
+        <v>Miercoles_Observaciones</v>
+      </c>
+      <c r="Y1" t="str">
         <v>Jueves_Tipo</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>Jueves_Cliente</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>Jueves_Inicio1</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>Jueves_Fin1</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>Jueves_Inicio2</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>Jueves_Fin2</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
+        <v>Jueves_Observaciones</v>
+      </c>
+      <c r="AF1" t="str">
         <v>Viernes_Tipo</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AG1" t="str">
         <v>Viernes_Cliente</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AH1" t="str">
         <v>Viernes_Inicio1</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AI1" t="str">
         <v>Viernes_Fin1</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AJ1" t="str">
         <v>Viernes_Inicio2</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AK1" t="str">
         <v>Viernes_Fin2</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AL1" t="str">
+        <v>Viernes_Observaciones</v>
+      </c>
+      <c r="AM1" t="str">
         <v>Sabado_Tipo</v>
       </c>
-      <c r="AI1" t="str">
+      <c r="AN1" t="str">
         <v>Sabado_Cliente</v>
       </c>
-      <c r="AJ1" t="str">
+      <c r="AO1" t="str">
         <v>Sabado_Inicio1</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AP1" t="str">
         <v>Sabado_Fin1</v>
       </c>
-      <c r="AL1" t="str">
+      <c r="AQ1" t="str">
         <v>Sabado_Inicio2</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AR1" t="str">
         <v>Sabado_Fin2</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AS1" t="str">
+        <v>Sabado_Observaciones</v>
+      </c>
+      <c r="AT1" t="str">
         <v>Domingo_Tipo</v>
       </c>
-      <c r="AO1" t="str">
+      <c r="AU1" t="str">
         <v>Domingo_Cliente</v>
       </c>
-      <c r="AP1" t="str">
+      <c r="AV1" t="str">
         <v>Domingo_Inicio1</v>
       </c>
-      <c r="AQ1" t="str">
+      <c r="AW1" t="str">
         <v>Domingo_Fin1</v>
       </c>
-      <c r="AR1" t="str">
+      <c r="AX1" t="str">
         <v>Domingo_Inicio2</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AY1" t="str">
         <v>Domingo_Fin2</v>
       </c>
-      <c r="AT1" t="str">
-        <v>Observaciones</v>
+      <c r="AZ1" t="str">
+        <v>Domingo_Observaciones</v>
+      </c>
+      <c r="BA1" t="str">
+        <v>Observaciones_Generales</v>
       </c>
     </row>
     <row r="2">
@@ -593,7 +621,7 @@
         <v>1017123456</v>
       </c>
       <c r="B2" t="str">
-        <v>Juan Camilo Lopez</v>
+        <v>Juan Camilo López</v>
       </c>
       <c r="C2" t="str">
         <v>2026-08-03</v>
@@ -617,115 +645,136 @@
         <v/>
       </c>
       <c r="J2" t="str">
+        <v>Llegar 10 min antes en sede principal</v>
+      </c>
+      <c r="K2" t="str">
         <v>Partido</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Almacenes Éxito S.A.</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>07:00</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>11:00</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>14:00</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>18:00</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
+        <v>Ruta express norte y llevar datáfono</v>
+      </c>
+      <c r="R2" t="str">
         <v>Continua</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="S2" t="str">
         <v>Droguerías Comfandi</v>
       </c>
-      <c r="R2" t="str">
+      <c r="T2" t="str">
         <v>07:00</v>
       </c>
-      <c r="S2" t="str">
+      <c r="U2" t="str">
         <v>15:00</v>
       </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
       <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v>Verificar sellos de seguridad de paquetes</v>
+      </c>
+      <c r="Y2" t="str">
         <v>Partido</v>
       </c>
-      <c r="W2" t="str">
+      <c r="Z2" t="str">
         <v>Droguerías Comfandi</v>
       </c>
-      <c r="X2" t="str">
+      <c r="AA2" t="str">
         <v>07:00</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="AB2" t="str">
         <v>11:00</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AC2" t="str">
         <v>14:00</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AD2" t="str">
         <v>18:00</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AE2" t="str">
+        <v>Priorizar entregas de farmacia</v>
+      </c>
+      <c r="AF2" t="str">
         <v>Continua</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AG2" t="str">
         <v>Almacenes Éxito S.A.</v>
       </c>
-      <c r="AD2" t="str">
+      <c r="AH2" t="str">
         <v>07:00</v>
       </c>
-      <c r="AE2" t="str">
+      <c r="AI2" t="str">
         <v>15:00</v>
       </c>
-      <c r="AF2" t="str">
-        <v/>
-      </c>
-      <c r="AG2" t="str">
-        <v/>
-      </c>
-      <c r="AH2" t="str">
+      <c r="AJ2" t="str">
+        <v/>
+      </c>
+      <c r="AK2" t="str">
+        <v/>
+      </c>
+      <c r="AL2" t="str">
+        <v>Revisar combustible antes de iniciar ruta</v>
+      </c>
+      <c r="AM2" t="str">
         <v>Continua</v>
       </c>
-      <c r="AI2" t="str">
+      <c r="AN2" t="str">
         <v>Almacenes Éxito S.A.</v>
       </c>
-      <c r="AJ2" t="str">
+      <c r="AO2" t="str">
         <v>08:00</v>
       </c>
-      <c r="AK2" t="str">
+      <c r="AP2" t="str">
         <v>13:00</v>
       </c>
-      <c r="AL2" t="str">
-        <v/>
-      </c>
-      <c r="AM2" t="str">
-        <v/>
-      </c>
-      <c r="AN2" t="str">
+      <c r="AQ2" t="str">
+        <v/>
+      </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v>Turno reforzado de fin de semana</v>
+      </c>
+      <c r="AT2" t="str">
         <v>Descanso</v>
       </c>
-      <c r="AO2" t="str">
-        <v/>
-      </c>
-      <c r="AP2" t="str">
-        <v/>
-      </c>
-      <c r="AQ2" t="str">
-        <v/>
-      </c>
-      <c r="AR2" t="str">
-        <v/>
-      </c>
-      <c r="AS2" t="str">
-        <v/>
-      </c>
-      <c r="AT2" t="str">
-        <v>Turno estándar Zona Norte</v>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
+      <c r="AY2" t="str">
+        <v/>
+      </c>
+      <c r="AZ2" t="str">
+        <v>Descanso dominical programado</v>
+      </c>
+      <c r="BA2" t="str">
+        <v>Cumplir con EPP y dotación al día</v>
       </c>
     </row>
     <row r="3">
@@ -733,7 +782,7 @@
         <v>1020456789</v>
       </c>
       <c r="B3" t="str">
-        <v>Andres Felipe Restrepo</v>
+        <v>Andrés Felipe Restrepo</v>
       </c>
       <c r="C3" t="str">
         <v>2026-08-03</v>
@@ -742,7 +791,7 @@
         <v>Partido</v>
       </c>
       <c r="E3" t="str">
-        <v>Mercado Libre Colombia</v>
+        <v>Droguerías Comfandi</v>
       </c>
       <c r="F3" t="str">
         <v>08:00</v>
@@ -757,135 +806,157 @@
         <v>19:00</v>
       </c>
       <c r="J3" t="str">
+        <v>Entrega de medicamentos refrigerados</v>
+      </c>
+      <c r="K3" t="str">
         <v>Continua</v>
       </c>
-      <c r="K3" t="str">
-        <v>Mercado Libre Colombia</v>
-      </c>
       <c r="L3" t="str">
+        <v>Droguerías Comfandi</v>
+      </c>
+      <c r="M3" t="str">
         <v>07:00</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>15:00</v>
       </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
       <c r="O3" t="str">
         <v/>
       </c>
       <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>Ruta centros comerciales sur</v>
+      </c>
+      <c r="R3" t="str">
         <v>Partido</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="S3" t="str">
         <v>Almacenes Éxito S.A.</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>08:00</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>12:00</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>15:00</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>19:00</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
+        <v>Cobro contraentrega con datáfono</v>
+      </c>
+      <c r="Y3" t="str">
         <v>Continua</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Z3" t="str">
         <v>Almacenes Éxito S.A.</v>
       </c>
-      <c r="X3" t="str">
+      <c r="AA3" t="str">
         <v>07:00</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AB3" t="str">
         <v>15:00</v>
       </c>
-      <c r="Z3" t="str">
-        <v/>
-      </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v>Apoyo en despacho sede central</v>
+      </c>
+      <c r="AF3" t="str">
         <v>Partido</v>
       </c>
-      <c r="AC3" t="str">
-        <v>Mercado Libre Colombia</v>
-      </c>
-      <c r="AD3" t="str">
+      <c r="AG3" t="str">
+        <v>Droguerías Comfandi</v>
+      </c>
+      <c r="AH3" t="str">
         <v>08:00</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AI3" t="str">
         <v>12:00</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AJ3" t="str">
         <v>15:00</v>
       </c>
-      <c r="AG3" t="str">
+      <c r="AK3" t="str">
         <v>19:00</v>
       </c>
-      <c r="AH3" t="str">
+      <c r="AL3" t="str">
+        <v>Verificar direcciones con cliente</v>
+      </c>
+      <c r="AM3" t="str">
         <v>Continua</v>
       </c>
-      <c r="AI3" t="str">
-        <v>Mercado Libre Colombia</v>
-      </c>
-      <c r="AJ3" t="str">
+      <c r="AN3" t="str">
+        <v>Droguerías Comfandi</v>
+      </c>
+      <c r="AO3" t="str">
         <v>08:00</v>
       </c>
-      <c r="AK3" t="str">
+      <c r="AP3" t="str">
         <v>14:00</v>
       </c>
-      <c r="AL3" t="str">
-        <v/>
-      </c>
-      <c r="AM3" t="str">
-        <v/>
-      </c>
-      <c r="AN3" t="str">
+      <c r="AQ3" t="str">
+        <v/>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3" t="str">
+        <v>Jornada continua fin de semana</v>
+      </c>
+      <c r="AT3" t="str">
         <v>Descanso</v>
       </c>
-      <c r="AO3" t="str">
-        <v/>
-      </c>
-      <c r="AP3" t="str">
-        <v/>
-      </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3" t="str">
-        <v/>
-      </c>
-      <c r="AS3" t="str">
-        <v/>
-      </c>
-      <c r="AT3" t="str">
-        <v>Turno estándar Zona Sur</v>
+      <c r="AU3" t="str">
+        <v/>
+      </c>
+      <c r="AV3" t="str">
+        <v/>
+      </c>
+      <c r="AW3" t="str">
+        <v/>
+      </c>
+      <c r="AX3" t="str">
+        <v/>
+      </c>
+      <c r="AY3" t="str">
+        <v/>
+      </c>
+      <c r="AZ3" t="str">
+        <v>Descanso dominical programado</v>
+      </c>
+      <c r="BA3" t="str">
+        <v>Turno semanal zona sur</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AT3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BA3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>INSTRUCCIONES DE CARGA MASIVA DE TURNOS - SERGEM MENSAJERIA S.A.S.</v>
+        <v>INSTRUCCIONES PARA LA CARGA MASIVA DE TURNOS - SERGEM MENSAJERÍA S.A.S.</v>
       </c>
     </row>
     <row r="2">
@@ -895,7 +966,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1. Tipos de Turno:</v>
+        <v>1. Tipos de Turno Válidos:</v>
       </c>
       <c r="B3" t="str">
         <v>Continua</v>
@@ -918,7 +989,7 @@
         <v>2. Formato de Horas:</v>
       </c>
       <c r="B4" t="str">
-        <v>HH:MM (ejemplo: 07:00, 15:00, 18:00)</v>
+        <v>HH:MM (Ej: 07:00, 15:00, 18:00)</v>
       </c>
     </row>
     <row r="5">
@@ -926,7 +997,7 @@
         <v>3. Turno Partido:</v>
       </c>
       <c r="B5" t="str">
-        <v>Diligencie HoraInicio1-HoraFin1 y HoraInicio2-HoraFin2</v>
+        <v>Diligenciar HoraInicio1 - HoraFin1 (mañana) y HoraInicio2 - HoraFin2 (tarde)</v>
       </c>
     </row>
     <row r="6">
@@ -934,7 +1005,7 @@
         <v>4. Turno Continuo:</v>
       </c>
       <c r="B6" t="str">
-        <v>Diligencie HoraInicio1 y HoraFin1</v>
+        <v>Diligenciar únicamente HoraInicio1 y HoraFin1</v>
       </c>
     </row>
     <row r="7">
@@ -942,47 +1013,103 @@
         <v>5. Descanso:</v>
       </c>
       <c r="B7" t="str">
-        <v>Escriba Descanso en la columna de Tipo.</v>
+        <v>Colocar "Descanso" en el campo Tipo. Los campos de hora y cliente pueden quedar vacíos.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>6. Columna de Observaciones / Recomendaciones en Cada Día:</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Cada día incluye su columna "[Día]_Observaciones" para añadir recomendaciones específicas (ej: llegar antes, ruta express, llevar datáfono, sede asignada, etc.).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CLIENTES FRECUENTES DE SERGEM:</v>
+        <v xml:space="preserve">   Estas observaciones son visibles en tiempo real para el repartidor y el jefe de zona.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Almacenes Éxito S.A.</v>
+        <v>7. Cédula del Repartidor:</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Si el repartidor ya existe en la plataforma, sus turnos se actualizarán automáticamente.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Droguerías Comfandi</v>
+        <v xml:space="preserve">   Si la cédula es nueva, el sistema registrará al repartidor automáticamente en el equipo.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Mercado Libre Colombia</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Postobón S.A.</v>
+        <v>LISTADO DE CLIENTES DISPONIBLES EN SERGEM:</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Nutresa Logistics</v>
+        <v>Código / ID</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Nombre del Cliente</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Ciudad / Sede</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>CLI-01</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Almacenes Éxito S.A.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Cali</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CLI-02</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Droguerías Comfandi</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Cali</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>CLI-03</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Mercado Libre Colombia</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Cali</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>CLI-04</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Postobón S.A.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Cali</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>